<commit_message>
feat(skills): import Skills Development inputs from workbook; leviable from H23; 20 points reachable; golden expectations extended
</commit_message>
<xml_diff>
--- a/test-fixtures/golden/golden-populated-workbook.xlsx
+++ b/test-fixtures/golden/golden-populated-workbook.xlsx
@@ -791,31 +791,31 @@
     <row r="2">
       <c r="O2">
         <f>SUM(O4:O575)</f>
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="P2">
         <f>SUM(P4:P575)</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="Q2">
         <f>SUM(Q4:Q575)</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="R2">
         <f>SUM(R4:R575)</f>
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="S2">
         <f>SUM(S4:S575)</f>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="T2">
         <f>SUM(T4:T575)</f>
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="U2">
         <f>SUM(U4:U575)</f>
-        <v>0</v>
+        <v>7000</v>
       </c>
       <c r="V2" t="str">
         <v xml:space="preserve">Sampled </v>
@@ -929,27 +929,27 @@
     <row r="2">
       <c r="P2">
         <f>SUM(P4:P586)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="Q2">
         <f>SUM(Q4:Q586)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R2">
         <f>SUM(R4:R586)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2">
         <f>SUM(S4:S586)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="T2">
         <f>SUM(T4:T586)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U2">
         <f>SUM(U4:U586)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="str">
         <v>Sampled Absorption</v>
@@ -1108,31 +1108,31 @@
     <row r="1">
       <c r="O1">
         <f>SUM(O3:O1048576)</f>
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="P1">
         <f>SUM(P3:P1048576)</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="Q1">
         <f>SUM(Q3:Q1048576)</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="R1">
         <f>SUM(R3:R1048576)</f>
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="S1">
         <f>SUM(S3:S1048576)</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="T1">
         <f>SUM(T3:T1048576)</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="U1">
         <f>SUM(U3:U1048576)</f>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="V1" t="str">
         <v xml:space="preserve">Sampled </v>
@@ -1333,61 +1333,97 @@
       <c r="A19" t="str">
         <v>MAR</v>
       </c>
+      <c r="B19">
+        <v>8000</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
         <v>APR</v>
       </c>
+      <c r="B20">
+        <v>8000</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
         <v>MAY</v>
       </c>
+      <c r="B21">
+        <v>8000</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
         <v>JUN</v>
       </c>
+      <c r="B22">
+        <v>8000</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
         <v>JUL</v>
       </c>
+      <c r="B23">
+        <v>8000</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
         <v>AUG</v>
       </c>
+      <c r="B24">
+        <v>8000</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
         <v>SEP</v>
       </c>
+      <c r="B25">
+        <v>8000</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
         <v>OCT</v>
       </c>
+      <c r="B26">
+        <v>8000</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
         <v>NOV</v>
       </c>
+      <c r="B27">
+        <v>8000</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
         <v>DEC</v>
       </c>
+      <c r="B28">
+        <v>8000</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
         <v>JAN</v>
       </c>
+      <c r="B29">
+        <v>8000</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
         <v>FEB</v>
       </c>
+      <c r="B30">
+        <v>12000</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1395,13 +1431,13 @@
       </c>
       <c r="B31">
         <f>SUM(B19:B30)</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="32">
       <c r="B32">
         <f>B31*100</f>
-        <v>0</v>
+        <v>10000000</v>
       </c>
     </row>
   </sheetData>
@@ -7569,30 +7605,30 @@
       </c>
       <c r="B23">
         <f>'Category A'!O2+'Category BCDE'!O2+'Category F&amp;G'!O1</f>
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="C23">
         <f>'Category A'!P2+'Category BCDE'!P2+'Category F&amp;G'!P1</f>
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="D23">
         <f>'Category A'!Q2+'Category BCDE'!Q2+'Category F&amp;G'!Q1</f>
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="E23">
         <f>'Category A'!R2+'Category BCDE'!R2+'Category F&amp;G'!R1</f>
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="F23">
         <f>'Category A'!S2+'Category BCDE'!S2+'Category F&amp;G'!S1</f>
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="G23">
         <f>'Category A'!T2+'Category BCDE'!T2+'Category F&amp;G'!T1</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="J23">
         <f>SUM(B23:G23)</f>
@@ -7864,30 +7900,30 @@
       </c>
       <c r="B52">
         <f>'Category A'!O2</f>
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="C52">
         <f>'Category A'!P2</f>
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="D52">
         <f>'Category A'!Q2</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="E52">
         <f>'Category A'!R2</f>
-        <v>0</v>
+        <v>45000</v>
       </c>
       <c r="F52">
         <f>'Category A'!S2</f>
-        <v>0</v>
+        <v>4500</v>
       </c>
       <c r="G52">
         <f>'Category A'!T2</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>10000000</v>
       </c>
     </row>
     <row r="53">
@@ -8151,30 +8187,30 @@
       </c>
       <c r="B81">
         <f>'Category BCD(Hcount)'!P2</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C81">
         <f>'Category BCD(Hcount)'!Q2</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D81">
         <f>'Category BCD(Hcount)'!R2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E81">
         <f>'Category BCD(Hcount)'!S2</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F81">
         <f>'Category BCD(Hcount)'!T2</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G81">
         <f>'Category BCD(Hcount)'!U2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H81">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="82">
@@ -8404,7 +8440,7 @@
       </c>
       <c r="B109">
         <f>'Category A'!U2+'Category BCDE'!U2+'Category F&amp;G'!U1</f>
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="D109">
         <f>B110*0.3%</f>
@@ -8417,7 +8453,7 @@
       </c>
       <c r="B110">
         <f>H23</f>
-        <v>0</v>
+        <v>10000000</v>
       </c>
     </row>
     <row r="111">
@@ -8436,7 +8472,7 @@
         <v xml:space="preserve">Completed Learners </v>
       </c>
       <c r="B115">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="116">
@@ -8444,7 +8480,7 @@
         <v xml:space="preserve">Total Headcount </v>
       </c>
       <c r="B116">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
   </sheetData>
@@ -8644,31 +8680,31 @@
     <row r="2">
       <c r="O2">
         <f>SUM(O4:O1048576)</f>
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="P2">
         <f>SUM(P4:P1048576)</f>
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="Q2">
         <f>SUM(Q4:Q1048576)</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="R2">
         <f>SUM(R4:R1048576)</f>
-        <v>0</v>
+        <v>45000</v>
       </c>
       <c r="S2">
         <f>SUM(S4:S1048576)</f>
-        <v>0</v>
+        <v>4500</v>
       </c>
       <c r="T2">
         <f>SUM(T4:T1048576)</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="U2">
         <f>SUM(U4:U1048576)</f>
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="V2" t="str">
         <v xml:space="preserve">Sampled </v>

</xml_diff>

<commit_message>
feat(mc): import MC scoring inputs from F/G block and Employment Equity; EAP surfaced not asserted; 19 points reachable; golden reaches Level 8
</commit_message>
<xml_diff>
--- a/test-fixtures/golden/golden-populated-workbook.xlsx
+++ b/test-fixtures/golden/golden-populated-workbook.xlsx
@@ -4550,7 +4550,7 @@
         <v>Black Board Members</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M4" t="str">
         <v>COR-39 - latest</v>
@@ -4578,7 +4578,7 @@
         <v>Total Board Members</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M5" t="str">
         <v>Management Organogram</v>
@@ -4611,7 +4611,7 @@
         <v>Black Female Board Members</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M7" t="str">
         <v xml:space="preserve">Latest minutes for board meetings </v>
@@ -4622,7 +4622,7 @@
         <v>Total Board Members</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M8" t="str">
         <v>EEA2 Forms and Proof of Submission</v>
@@ -4655,7 +4655,7 @@
         <v>Black Executive Directors</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M10" t="str">
         <v>Acknowlegement Letter</v>
@@ -4683,7 +4683,7 @@
         <v xml:space="preserve">Total Executive Directors </v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -4694,7 +4694,7 @@
         <v>Black Female Executive Directors</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -4719,7 +4719,7 @@
         <v>Total Executive Directors</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -4744,7 +4744,7 @@
         <v>Black Executive Management</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
@@ -4752,7 +4752,7 @@
         <v>Total Executive Management</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
@@ -4770,7 +4770,7 @@
         <v>Black Executive Management</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20">
@@ -4778,7 +4778,7 @@
         <v>Total Executive Management</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -5566,31 +5566,25 @@
         <v xml:space="preserve">Total employees per race </v>
       </c>
       <c r="B29">
-        <f>'5 Staff List '!L2</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C29">
-        <f>'5 Staff List '!M2</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D29">
-        <f>'5 Staff List '!N2</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E29">
-        <f>'5 Staff List '!O2</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F29">
-        <f>'5 Staff List '!P2</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G29">
-        <f>'5 Staff List '!Q2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30">
@@ -5853,20 +5847,16 @@
         <v xml:space="preserve">Total employees per race </v>
       </c>
       <c r="E58">
-        <f>'5 Staff List '!O2</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F58">
-        <f>'5 Staff List '!P2</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G58">
-        <f>'5 Staff List '!Q2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H58">
-        <f>H29</f>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="59">
@@ -6063,31 +6053,25 @@
         <v xml:space="preserve">Total employees per race </v>
       </c>
       <c r="B87">
-        <f>'5 Staff List '!R2</f>
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="C87">
-        <f>'5 Staff List '!S2</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D87">
-        <f>'5 Staff List '!T2</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E87">
-        <f>'5 Staff List '!U2</f>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="F87">
-        <f>'5 Staff List '!V2</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G87">
-        <f>'5 Staff List '!W2</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H87">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="88">
@@ -6350,20 +6334,16 @@
         <v xml:space="preserve">Total employees per race </v>
       </c>
       <c r="E118">
-        <f>'5 Staff List '!U2</f>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="F118">
-        <f>'5 Staff List '!V2</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G118">
-        <f>'5 Staff List '!W2</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H118">
-        <f>H87</f>
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="119">
@@ -6560,31 +6540,25 @@
         <v xml:space="preserve">Total employees per race </v>
       </c>
       <c r="B147">
-        <f>'5 Staff List '!X2</f>
-        <v>0</v>
+        <v>330</v>
       </c>
       <c r="C147">
-        <f>'5 Staff List '!Y2</f>
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="D147">
-        <f>'5 Staff List '!Z2</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E147">
-        <f>'5 Staff List '!AA2</f>
-        <v>0</v>
+        <v>290</v>
       </c>
       <c r="F147">
-        <f>'5 Staff List '!AB2</f>
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G147">
-        <f>'5 Staff List '!AC2</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H147">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="148">
@@ -6847,20 +6821,16 @@
         <v xml:space="preserve">Total employees per race </v>
       </c>
       <c r="E176">
-        <f>'5 Staff List '!AA2</f>
-        <v>0</v>
+        <v>290</v>
       </c>
       <c r="F176">
-        <f>'5 Staff List '!AB2</f>
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G176">
-        <f>'5 Staff List '!AC2</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H176">
-        <f>H147</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="177">
@@ -7023,7 +6993,7 @@
         <v xml:space="preserve">Black </v>
       </c>
       <c r="B204">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="205">
@@ -7031,7 +7001,7 @@
         <v xml:space="preserve">Total </v>
       </c>
       <c r="B205">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(closers): new-entrants import (25/25 reachable), pending_confirmation status, rule_set_snapshot persisted and honoured, phantom-key sweep
</commit_message>
<xml_diff>
--- a/test-fixtures/golden/golden-populated-workbook.xlsx
+++ b/test-fixtures/golden/golden-populated-workbook.xlsx
@@ -2656,7 +2656,7 @@
       </c>
       <c r="D10">
         <f>K22</f>
-        <v>0.065</v>
+        <v>0.013</v>
       </c>
       <c r="E10">
         <f>IF(C10=0,0,MIN(D10/C10*B10,B10))</f>
@@ -2772,7 +2772,7 @@
         <v>0.03</v>
       </c>
       <c r="G17">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="H17">
         <f>$C$17*D17</f>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="K17">
         <f>$C$17*G17</f>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="18">
@@ -2811,7 +2811,7 @@
         <v>0.02</v>
       </c>
       <c r="G18">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="H18">
         <f>$C$18*D18</f>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="K18">
         <f>$C$18*G18</f>
-        <v>0.015</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="19">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="K22">
         <f>SUM(K17:K21)</f>
-        <v>0.065</v>
+        <v>0.013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>